<commit_message>
update-olap-excel: Updated Data Dictionary and ETL Mapping to align with develop changes, including data types and constraints adjustments
</commit_message>
<xml_diff>
--- a/docs/olap/Senior Care Management - Data Dictionary.xlsx
+++ b/docs/olap/Senior Care Management - Data Dictionary.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visit" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Senior" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CareGiver" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agency" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP DimDate" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP DimSenior" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP DimProfessional" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP DimService" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP DimOrganization" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OLAP FactVisit" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Visit" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Person" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Senior" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CareGiver" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Agency" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Service" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="OLAP DimDate" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="OLAP DimSenior" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="OLAP DimProfessional" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="OLAP DimService" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="OLAP DimOrganization" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="OLAP FactVisit" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -856,6 +858,298 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Nullability</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Key / Relationship</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>DimService</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>ServiceKey</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>int IDENTITY</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Warehouse surrogate key</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>DimService</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>ServiceID</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>UNIQUE; Service.ServiceID</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Natural key</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>DimService</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>ServiceName</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>nvarchar(100)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>From OLTP Service</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Nullability</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Key / Relationship</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>DimOrganization</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>OrganizationKey</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>int IDENTITY</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Warehouse surrogate key</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>DimOrganization</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>OrganizationID</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>UNIQUE; Agency.AgencyID</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Natural key</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>DimOrganization</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>OrganizationName</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>nvarchar(200)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>From Agency.Name</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1321,6 +1615,358 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="18.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8.21875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="35" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="8.109375" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Allowed Values/Rules</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Sensitive</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>PersonID</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Primary key, unique</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>FirstName</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>MiddleName</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>LastName</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Street</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(200)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Province</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>PostalCode</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Shared details</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Names, address and phone for Seniors, Caregivers, Family Members and Agency Managers live here; SeniorID, CaregiverID, FamilyMemberID and AgencyManagerID equal PersonID. Login email is on the user account (AspNetUsers).</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="32" customHeight="1"/>
+    <row r="15" ht="32" customHeight="1"/>
+    <row r="16" ht="32" customHeight="1"/>
+    <row r="17" ht="32" customHeight="1"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1699,7 +2345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1838,11 +2484,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="2" t="n"/>
@@ -1867,7 +2508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2171,7 +2812,149 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="18.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8.21875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="35" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="8.109375" bestFit="1" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Allowed Values/Rules</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Sensitive</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>ServiceID</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Primary key, unique</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>ServiceName</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Cannot be empty; seeded as Doctor, Home visit, Bathing (OLTP-16)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1"/>
+    <row r="6" ht="32" customHeight="1"/>
+    <row r="7" ht="32" customHeight="1"/>
+    <row r="8" ht="32" customHeight="1"/>
+    <row r="9" ht="32" customHeight="1"/>
+    <row r="10" ht="32" customHeight="1"/>
+    <row r="11" ht="32" customHeight="1"/>
+    <row r="12" ht="32" customHeight="1"/>
+    <row r="13" ht="32" customHeight="1"/>
+    <row r="14" ht="32" customHeight="1"/>
+    <row r="15" ht="32" customHeight="1"/>
+    <row r="16" ht="32" customHeight="1"/>
+    <row r="17" ht="32" customHeight="1"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2429,7 +3212,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2687,7 +3470,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2859,296 +3642,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Nullability</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Key / Relationship</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>DimService</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>ServiceKey</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>int IDENTITY</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Warehouse surrogate key</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>DimService</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>ServiceID</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>UNIQUE; Service.ServiceID</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Natural key</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>DimService</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>ServiceName</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>nvarchar(100)</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>From OLTP Service</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Nullability</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Key / Relationship</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>DimOrganization</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>OrganizationKey</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>int IDENTITY</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Warehouse surrogate key</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>DimOrganization</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>OrganizationID</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>UNIQUE; Agency.AgencyID</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Natural key</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>DimOrganization</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>OrganizationName</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>nvarchar(200)</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>From Agency.Name</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>